<commit_message>
Adicionando força de trabalho
</commit_message>
<xml_diff>
--- a/calculo_estatistica_educacao/estatistica_populacional_brasil.xlsx
+++ b/calculo_estatistica_educacao/estatistica_populacional_brasil.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gisel\PycharmProjects\Tcc_demografia\calculo_estatistica_educacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E95560C-B1E6-4759-8021-1B17D4589C39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20335A51-9ACE-4665-AFE8-C603C5F3B9F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -426,7 +426,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -456,10 +456,6 @@
     <xf numFmtId="43" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -832,16 +828,16 @@
     <row r="1" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11"/>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
       <c r="J2" s="10"/>
       <c r="M2" s="6" t="s">
         <v>2</v>
@@ -891,7 +887,7 @@
     </row>
     <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="11"/>
-      <c r="B4" s="39" t="s">
+      <c r="B4" s="35" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -927,7 +923,7 @@
     </row>
     <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="11"/>
-      <c r="B5" s="37"/>
+      <c r="B5" s="33"/>
       <c r="C5" s="6" t="s">
         <v>8</v>
       </c>
@@ -961,7 +957,7 @@
     </row>
     <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="32" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -997,7 +993,7 @@
     </row>
     <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
-      <c r="B7" s="37"/>
+      <c r="B7" s="33"/>
       <c r="C7" s="6" t="s">
         <v>8</v>
       </c>
@@ -1031,7 +1027,7 @@
     </row>
     <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="32" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="6" t="s">
@@ -1067,7 +1063,7 @@
     </row>
     <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
-      <c r="B9" s="37"/>
+      <c r="B9" s="33"/>
       <c r="C9" s="6" t="s">
         <v>8</v>
       </c>
@@ -1092,7 +1088,7 @@
     </row>
     <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="11"/>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="32" t="s">
         <v>11</v>
       </c>
       <c r="C10" s="6" t="s">
@@ -1119,7 +1115,7 @@
     </row>
     <row r="11" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11"/>
-      <c r="B11" s="38"/>
+      <c r="B11" s="34"/>
       <c r="C11" s="8" t="s">
         <v>8</v>
       </c>
@@ -1144,16 +1140,16 @@
     </row>
     <row r="15" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="31"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="31"/>
-      <c r="I16" s="33"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="29"/>
     </row>
     <row r="17" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
@@ -1182,301 +1178,301 @@
       </c>
     </row>
     <row r="18" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B18" s="34" t="s">
+      <c r="B18" s="30" t="s">
         <v>6</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="17">
+      <c r="D18" s="18">
         <f>21998353.26/N3</f>
         <v>0.41625572862321292</v>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="18">
         <f>23527608.37/N4</f>
         <v>0.57392885725989073</v>
       </c>
-      <c r="F18" s="22">
+      <c r="F18" s="18">
         <f>21674503.19/N5</f>
         <v>0.66819687443250064</v>
       </c>
-      <c r="G18" s="22">
+      <c r="G18" s="18">
         <f>18772868/N6</f>
         <v>0.78912268302085498</v>
       </c>
-      <c r="H18" s="22">
+      <c r="H18" s="18">
         <f>15798899/N7</f>
         <v>0.88166081874608493</v>
       </c>
-      <c r="I18" s="26">
+      <c r="I18" s="22">
         <f>13234705/N8</f>
         <v>0.92796782786181209</v>
       </c>
     </row>
     <row r="19" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B19" s="35"/>
+      <c r="B19" s="31"/>
       <c r="C19" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D19" s="18">
+      <c r="D19" s="19">
         <f>22999117.77/O3</f>
         <v>0.39829299617035224</v>
       </c>
-      <c r="E19" s="23">
+      <c r="E19" s="19">
         <f>25134670.61/O4</f>
         <v>0.56512862246772733</v>
       </c>
-      <c r="F19" s="23">
+      <c r="F19" s="19">
         <f>23574787.07/O5</f>
         <v>0.67730729621321739</v>
       </c>
-      <c r="G19" s="23">
+      <c r="G19" s="19">
         <f>19941339/O6</f>
         <v>0.80959653376290219</v>
       </c>
-      <c r="H19" s="23">
+      <c r="H19" s="19">
         <f>16235597/O7</f>
         <v>0.90431224388741382</v>
       </c>
-      <c r="I19" s="27">
+      <c r="I19" s="23">
         <f>13338845/O8</f>
         <v>0.94681646212051307</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="20">
         <f>12983965.13/N3</f>
         <v>0.24568429289813756</v>
       </c>
-      <c r="E20" s="24">
+      <c r="E20" s="20">
         <f>8278710.12/N4</f>
         <v>0.20194958042637176</v>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="20">
         <f>5025392.11/N5</f>
         <v>0.15492633308656473</v>
       </c>
-      <c r="G20" s="24">
+      <c r="G20" s="20">
         <f>2444182/N6</f>
         <v>0.10274186435611647</v>
       </c>
-      <c r="H20" s="24">
+      <c r="H20" s="20">
         <f>1106541/N7</f>
         <v>6.1750748836112666E-2</v>
       </c>
-      <c r="I20" s="26">
+      <c r="I20" s="22">
         <f>527400/N8</f>
         <v>3.6979307994724452E-2</v>
       </c>
     </row>
     <row r="21" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B21" s="35"/>
+      <c r="B21" s="31"/>
       <c r="C21" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="18">
+      <c r="D21" s="19">
         <f>13228057.92/O3</f>
         <v>0.22908021408300122</v>
       </c>
-      <c r="E21" s="23">
+      <c r="E21" s="19">
         <f>8504580.79/O4</f>
         <v>0.19121722743428449</v>
       </c>
-      <c r="F21" s="23">
+      <c r="F21" s="19">
         <f>4959499.87/O5</f>
         <v>0.1424872020071867</v>
       </c>
-      <c r="G21" s="23">
+      <c r="G21" s="19">
         <f>2221557/O6</f>
         <v>9.0192782277895775E-2</v>
       </c>
-      <c r="H21" s="23">
+      <c r="H21" s="19">
         <f>902268/O7</f>
         <v>5.0255743578003879E-2</v>
       </c>
-      <c r="I21" s="27">
+      <c r="I21" s="23">
         <f>490030/O8</f>
         <v>3.4783256791192568E-2</v>
       </c>
     </row>
     <row r="22" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="25" t="s">
         <v>10</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="20">
         <f>12609168.91/N3</f>
         <v>0.23859234961504627</v>
       </c>
-      <c r="E22" s="24">
+      <c r="E22" s="20">
         <f>6583473.61/N4</f>
         <v>0.1605962419285181</v>
       </c>
-      <c r="F22" s="24">
+      <c r="F22" s="20">
         <f>3823758.48/N5</f>
         <v>0.11788152385885295</v>
       </c>
-      <c r="G22" s="24">
+      <c r="G22" s="20">
         <f>1610328/N6</f>
         <v>6.7690581529876379E-2</v>
       </c>
-      <c r="H22" s="24">
+      <c r="H22" s="20">
         <f>604708/N7</f>
         <v>3.3745854719516057E-2</v>
       </c>
-      <c r="I22" s="26">
+      <c r="I22" s="22">
         <f>292660/N8</f>
         <v>2.0520220473523053E-2</v>
       </c>
     </row>
     <row r="23" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B23" s="35"/>
+      <c r="B23" s="31"/>
       <c r="C23" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D23" s="18">
+      <c r="D23" s="19">
         <f>14311194.33/O3</f>
         <v>0.24783770079681003</v>
       </c>
-      <c r="E23" s="23">
+      <c r="E23" s="19">
         <f>7982454.4/O4</f>
         <v>0.17947772337977932</v>
       </c>
-      <c r="F23" s="23">
+      <c r="F23" s="19">
         <f>4491542.2/O5</f>
         <v>0.12904270542408619</v>
       </c>
-      <c r="G23" s="23">
+      <c r="G23" s="19">
         <f>1838099/O6</f>
         <v>7.4624807246547326E-2</v>
       </c>
-      <c r="H23" s="23">
+      <c r="H23" s="19">
         <f>692003/O7</f>
         <v>3.8544119178791025E-2</v>
       </c>
-      <c r="I23" s="27">
+      <c r="I23" s="23">
         <f>230415/O8</f>
         <v>1.6355292764815694E-2</v>
       </c>
     </row>
     <row r="24" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B24" s="29" t="s">
+      <c r="B24" s="25" t="s">
         <v>11</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="20">
         <f>5256682.1/N3</f>
         <v>9.9467628863602511E-2</v>
       </c>
-      <c r="E24" s="24">
+      <c r="E24" s="20">
         <f>2604153.53/N4</f>
         <v>6.3525320385219006E-2</v>
       </c>
-      <c r="F24" s="24">
+      <c r="F24" s="20">
         <f>1913647.29/N5</f>
         <v>5.8995268622082084E-2</v>
       </c>
-      <c r="G24" s="24">
+      <c r="G24" s="20">
         <f>962165/N6</f>
         <v>4.0444871093152146E-2</v>
       </c>
-      <c r="H24" s="24">
+      <c r="H24" s="20">
         <f>409327/N7</f>
         <v>2.2842577698286362E-2</v>
       </c>
-      <c r="I24" s="26">
+      <c r="I24" s="22">
         <f>207265/N8</f>
         <v>1.4532643669940394E-2</v>
       </c>
     </row>
     <row r="25" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="30"/>
+      <c r="B25" s="26"/>
       <c r="C25" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="21">
         <f>7205848.41/O3</f>
         <v>0.12478908894983536</v>
       </c>
-      <c r="E25" s="25">
+      <c r="E25" s="21">
         <f>2854311.89/O4</f>
         <v>6.4176426718207766E-2</v>
       </c>
-      <c r="F25" s="25">
+      <c r="F25" s="21">
         <f>1780804.72/O5</f>
         <v>5.1162796355510645E-2</v>
       </c>
-      <c r="G25" s="25">
+      <c r="G25" s="21">
         <f>630211/O6</f>
         <v>2.5585876712654672E-2</v>
       </c>
-      <c r="H25" s="25">
+      <c r="H25" s="21">
         <f>123662/O7</f>
         <v>6.8878933557913122E-3</v>
       </c>
-      <c r="I25" s="28">
+      <c r="I25" s="24">
         <f>28810/O8</f>
         <v>2.0449883234786807E-3</v>
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D26" s="21">
+      <c r="D26" s="17">
         <f>SUM(D18,D20,D22,D24)</f>
         <v>0.99999999999999922</v>
       </c>
-      <c r="E26" s="21">
+      <c r="E26" s="17">
         <f t="shared" ref="E26:I26" si="0">SUM(E18,E20,E22,E24)</f>
         <v>0.99999999999999956</v>
       </c>
-      <c r="F26" s="21">
+      <c r="F26" s="17">
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G26" s="21">
+      <c r="G26" s="17">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H26" s="21">
+      <c r="H26" s="17">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="I26" s="21">
+      <c r="I26" s="17">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D27" s="21">
+      <c r="D27" s="17">
         <f>SUM(D19,D21,D23,D25)</f>
         <v>0.99999999999999878</v>
       </c>
-      <c r="E27" s="21">
+      <c r="E27" s="17">
         <f t="shared" ref="E27:I27" si="1">SUM(E19,E21,E23,E25)</f>
         <v>0.99999999999999889</v>
       </c>
-      <c r="F27" s="21">
+      <c r="F27" s="17">
         <f t="shared" si="1"/>
         <v>1.0000000000000009</v>
       </c>
-      <c r="G27" s="21">
+      <c r="G27" s="17">
         <f t="shared" si="1"/>
         <v>0.99999999999999989</v>
       </c>
-      <c r="H27" s="21">
+      <c r="H27" s="17">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="I27" s="21">
+      <c r="I27" s="17">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>

</xml_diff>